<commit_message>
found a new output method and it works, the solution also works but for some reason the output is mirrored. need to fix that
</commit_message>
<xml_diff>
--- a/ARC_input1.xlsx
+++ b/ARC_input1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\malis\ARC_PROJECT\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1DE628B7-FCE7-423B-A414-A11F78611018}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6ACD5553-47D0-4B76-B1F6-5C22CE1FE868}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="8490" yWindow="5535" windowWidth="28800" windowHeight="15345" xr2:uid="{F53C116B-94EC-42D2-B4AD-E1458F2C02A3}"/>
+    <workbookView xWindow="40230" yWindow="4170" windowWidth="28800" windowHeight="15345" xr2:uid="{F53C116B-94EC-42D2-B4AD-E1458F2C02A3}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -29,7 +29,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -54,14 +54,8 @@
         <bgColor rgb="FF0070C0"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="2">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -84,17 +78,60 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" customBuiltin="1"/>
@@ -541,7 +578,7 @@
       <c r="G9" s="2"/>
       <c r="H9" s="2"/>
       <c r="I9" s="2"/>
-      <c r="J9" s="2"/>
+      <c r="J9" s="6"/>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A10" s="2"/>
@@ -549,11 +586,11 @@
       <c r="C10" s="2"/>
       <c r="D10" s="2"/>
       <c r="E10" s="2"/>
-      <c r="F10" s="5"/>
+      <c r="F10" s="2"/>
       <c r="G10" s="2"/>
       <c r="H10" s="2"/>
-      <c r="I10" s="2"/>
-      <c r="J10" s="2"/>
+      <c r="I10" s="5"/>
+      <c r="J10" s="7"/>
     </row>
   </sheetData>
   <pageMargins left="0.70000000000000007" right="0.70000000000000007" top="0.75" bottom="0.75" header="0.30000000000000004" footer="0.30000000000000004"/>

</xml_diff>

<commit_message>
finally managed to make it work correctly. the code can be cleaner and clearer. i'll take a look once again before the meeting.
</commit_message>
<xml_diff>
--- a/ARC_input1.xlsx
+++ b/ARC_input1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\malis\ARC_PROJECT\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6ACD5553-47D0-4B76-B1F6-5C22CE1FE868}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{30CD3577-05FF-4C52-BCBB-167FEBDF41EA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="40230" yWindow="4170" windowWidth="28800" windowHeight="15345" xr2:uid="{F53C116B-94EC-42D2-B4AD-E1458F2C02A3}"/>
+    <workbookView xWindow="6225" yWindow="3105" windowWidth="28800" windowHeight="15345" xr2:uid="{F53C116B-94EC-42D2-B4AD-E1458F2C02A3}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -29,7 +29,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -54,6 +54,12 @@
         <bgColor rgb="FF0070C0"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
+        <bgColor rgb="FFD86DCD"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="5">
     <border>
@@ -123,7 +129,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
@@ -132,6 +138,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" customBuiltin="1"/>
@@ -476,7 +483,7 @@
       <c r="A1" s="1"/>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
-      <c r="D1" s="1"/>
+      <c r="D1" s="8"/>
       <c r="E1" s="2"/>
       <c r="F1" s="2"/>
       <c r="G1" s="2"/>
@@ -516,7 +523,7 @@
       <c r="E4" s="2"/>
       <c r="F4" s="2"/>
       <c r="G4" s="2"/>
-      <c r="H4" s="1"/>
+      <c r="H4" s="8"/>
       <c r="I4" s="2"/>
       <c r="J4" s="2"/>
     </row>

</xml_diff>